<commit_message>
Actualización automática desde SharePoint
</commit_message>
<xml_diff>
--- a/Base_Dato_Indisponibilidad_GEN_CL.xlsx
+++ b/Base_Dato_Indisponibilidad_GEN_CL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie.sharepoint.com/sites/OperacionesCentralMejillones-Administracin/Shared Documents/Administración/0.- Gerencia/02.- Operación/05.- EFOF_GEN_CL/05.- PRO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="850" documentId="8_{55EF2082-D0B7-4F26-90F5-434FA2717943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B96CBE0-23B9-4030-928F-6EFE6EE0E5ED}"/>
+  <xr:revisionPtr revIDLastSave="853" documentId="8_{55EF2082-D0B7-4F26-90F5-434FA2717943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E9DF501-2FF6-4289-B146-A361D0BE00CF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{E052323F-F4D0-446A-B69C-8F538CB3C6F5}"/>
+    <workbookView xWindow="-25935" yWindow="5655" windowWidth="21600" windowHeight="11085" firstSheet="2" activeTab="2" xr2:uid="{E052323F-F4D0-446A-B69C-8F538CB3C6F5}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DATOS_EVENTOS_GEN_CHILE" sheetId="1" r:id="rId1"/>
@@ -273,7 +273,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -361,10 +361,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ h:mm"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ h:mm"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -373,11 +373,11 @@
       <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ h:mm"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ h:mm"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1069,8 +1069,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE341A5-48DC-491A-A7A3-9CB9E0074F67}">
-  <dimension ref="A9:I331"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:I331"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -1084,13 +1084,18 @@
     <col min="12" max="12" width="33.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9">
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" s="2">
         <f>SUBTOTAL(103,BD_GEN_CL[Unidad])</f>
         <v>298</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -1119,7 +1124,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9">
       <c r="A11" s="1">
         <v>1</v>
       </c>
@@ -1145,7 +1150,7 @@
       <c r="H11" s="11"/>
       <c r="I11" s="11"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9">
       <c r="A12" s="1">
         <v>2</v>
       </c>
@@ -1171,7 +1176,7 @@
       <c r="H12" s="11"/>
       <c r="I12" s="11"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
       <c r="A13" s="1">
         <v>3</v>
       </c>
@@ -1197,7 +1202,7 @@
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9">
       <c r="A14" s="1">
         <v>4</v>
       </c>
@@ -1223,7 +1228,7 @@
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9">
       <c r="A15" s="1">
         <v>5</v>
       </c>
@@ -1249,7 +1254,7 @@
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9">
       <c r="A16" s="1">
         <v>6</v>
       </c>
@@ -1275,7 +1280,7 @@
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9">
       <c r="A17" s="1">
         <v>7</v>
       </c>
@@ -1301,7 +1306,7 @@
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9">
       <c r="A18" s="1">
         <v>8</v>
       </c>
@@ -1327,7 +1332,7 @@
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9">
       <c r="A19" s="1">
         <v>9</v>
       </c>
@@ -1353,7 +1358,7 @@
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9">
       <c r="A20" s="1">
         <v>10</v>
       </c>
@@ -1379,7 +1384,7 @@
       <c r="H20" s="11"/>
       <c r="I20" s="11"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9">
       <c r="A21" s="1">
         <v>11</v>
       </c>
@@ -1405,7 +1410,7 @@
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9">
       <c r="A22" s="1">
         <v>12</v>
       </c>
@@ -1431,7 +1436,7 @@
       <c r="H22" s="11"/>
       <c r="I22" s="11"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9">
       <c r="A23" s="1">
         <v>13</v>
       </c>
@@ -1457,7 +1462,7 @@
       <c r="H23" s="11"/>
       <c r="I23" s="11"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9">
       <c r="A24" s="1">
         <v>14</v>
       </c>
@@ -1483,7 +1488,7 @@
       <c r="H24" s="11"/>
       <c r="I24" s="11"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9">
       <c r="A25" s="1">
         <v>15</v>
       </c>
@@ -1509,7 +1514,7 @@
       <c r="H25" s="11"/>
       <c r="I25" s="11"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9">
       <c r="A26" s="1">
         <v>16</v>
       </c>
@@ -1535,7 +1540,7 @@
       <c r="H26" s="11"/>
       <c r="I26" s="11"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9">
       <c r="A27" s="1">
         <v>17</v>
       </c>
@@ -1561,7 +1566,7 @@
       <c r="H27" s="11"/>
       <c r="I27" s="11"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9">
       <c r="A28" s="1">
         <v>18</v>
       </c>
@@ -1587,7 +1592,7 @@
       <c r="H28" s="11"/>
       <c r="I28" s="11"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9">
       <c r="A29" s="1">
         <v>19</v>
       </c>
@@ -1613,7 +1618,7 @@
       <c r="H29" s="11"/>
       <c r="I29" s="11"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9">
       <c r="A30" s="1">
         <v>20</v>
       </c>
@@ -1639,7 +1644,7 @@
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9">
       <c r="A31" s="1">
         <v>21</v>
       </c>
@@ -1665,7 +1670,7 @@
       <c r="H31" s="11"/>
       <c r="I31" s="11"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9">
       <c r="A32" s="1">
         <v>22</v>
       </c>
@@ -1691,7 +1696,7 @@
       <c r="H32" s="11"/>
       <c r="I32" s="11"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9">
       <c r="A33" s="1">
         <v>23</v>
       </c>
@@ -1717,7 +1722,7 @@
       <c r="H33" s="11"/>
       <c r="I33" s="11"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9">
       <c r="A34" s="1">
         <v>24</v>
       </c>
@@ -1743,7 +1748,7 @@
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9">
       <c r="A35" s="1">
         <v>25</v>
       </c>
@@ -1769,7 +1774,7 @@
       <c r="H35" s="11"/>
       <c r="I35" s="11"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9">
       <c r="A36" s="1">
         <v>26</v>
       </c>
@@ -1795,7 +1800,7 @@
       <c r="H36" s="11"/>
       <c r="I36" s="11"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9">
       <c r="A37" s="1">
         <v>27</v>
       </c>
@@ -1821,7 +1826,7 @@
       <c r="H37" s="11"/>
       <c r="I37" s="11"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9">
       <c r="A38" s="1">
         <v>28</v>
       </c>
@@ -1847,7 +1852,7 @@
       <c r="H38" s="11"/>
       <c r="I38" s="11"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9">
       <c r="A39" s="1">
         <v>29</v>
       </c>
@@ -1873,7 +1878,7 @@
       <c r="H39" s="11"/>
       <c r="I39" s="11"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9">
       <c r="A40" s="1">
         <v>30</v>
       </c>
@@ -1899,7 +1904,7 @@
       <c r="H40" s="11"/>
       <c r="I40" s="11"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9">
       <c r="A41" s="1">
         <v>31</v>
       </c>
@@ -1925,7 +1930,7 @@
       <c r="H41" s="11"/>
       <c r="I41" s="11"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9">
       <c r="A42" s="1">
         <v>32</v>
       </c>
@@ -1951,7 +1956,7 @@
       <c r="H42" s="11"/>
       <c r="I42" s="11"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9">
       <c r="A43" s="1">
         <v>33</v>
       </c>
@@ -1977,7 +1982,7 @@
       <c r="H43" s="11"/>
       <c r="I43" s="11"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9">
       <c r="A44" s="1">
         <v>34</v>
       </c>
@@ -2003,7 +2008,7 @@
       <c r="H44" s="11"/>
       <c r="I44" s="11"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9">
       <c r="A45" s="1">
         <v>35</v>
       </c>
@@ -2029,7 +2034,7 @@
       <c r="H45" s="11"/>
       <c r="I45" s="11"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9">
       <c r="A46" s="1">
         <v>36</v>
       </c>
@@ -2055,7 +2060,7 @@
       <c r="H46" s="11"/>
       <c r="I46" s="11"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9">
       <c r="A47" s="1">
         <v>37</v>
       </c>
@@ -2081,7 +2086,7 @@
       <c r="H47" s="11"/>
       <c r="I47" s="11"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9">
       <c r="A48" s="1">
         <v>38</v>
       </c>
@@ -2107,7 +2112,7 @@
       <c r="H48" s="11"/>
       <c r="I48" s="11"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9">
       <c r="A49" s="1">
         <v>39</v>
       </c>
@@ -2133,7 +2138,7 @@
       <c r="H49" s="11"/>
       <c r="I49" s="11"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9">
       <c r="A50" s="1">
         <v>40</v>
       </c>
@@ -2159,7 +2164,7 @@
       <c r="H50" s="11"/>
       <c r="I50" s="11"/>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9">
       <c r="A51" s="1">
         <v>41</v>
       </c>
@@ -2185,7 +2190,7 @@
       <c r="H51" s="11"/>
       <c r="I51" s="11"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9">
       <c r="A52" s="1">
         <v>42</v>
       </c>
@@ -2211,7 +2216,7 @@
       <c r="H52" s="11"/>
       <c r="I52" s="11"/>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9">
       <c r="A53" s="1">
         <v>43</v>
       </c>
@@ -2237,7 +2242,7 @@
       <c r="H53" s="11"/>
       <c r="I53" s="11"/>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9">
       <c r="A54" s="1">
         <v>44</v>
       </c>
@@ -2263,7 +2268,7 @@
       <c r="H54" s="11"/>
       <c r="I54" s="11"/>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9">
       <c r="A55" s="1">
         <v>45</v>
       </c>
@@ -2289,7 +2294,7 @@
       <c r="H55" s="11"/>
       <c r="I55" s="11"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9">
       <c r="A56" s="1">
         <v>46</v>
       </c>
@@ -2315,7 +2320,7 @@
       <c r="H56" s="11"/>
       <c r="I56" s="11"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9">
       <c r="A57" s="1">
         <v>47</v>
       </c>
@@ -2341,7 +2346,7 @@
       <c r="H57" s="11"/>
       <c r="I57" s="11"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9">
       <c r="A58" s="1">
         <v>48</v>
       </c>
@@ -2367,7 +2372,7 @@
       <c r="H58" s="11"/>
       <c r="I58" s="11"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9">
       <c r="A59" s="1">
         <v>49</v>
       </c>
@@ -2393,7 +2398,7 @@
       <c r="H59" s="11"/>
       <c r="I59" s="11"/>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9">
       <c r="A60" s="1">
         <v>50</v>
       </c>
@@ -2419,7 +2424,7 @@
       <c r="H60" s="11"/>
       <c r="I60" s="11"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9">
       <c r="A61" s="1">
         <v>51</v>
       </c>
@@ -2445,7 +2450,7 @@
       <c r="H61" s="11"/>
       <c r="I61" s="11"/>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9">
       <c r="A62" s="1">
         <v>52</v>
       </c>
@@ -2471,7 +2476,7 @@
       <c r="H62" s="11"/>
       <c r="I62" s="11"/>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9">
       <c r="A63" s="1">
         <v>53</v>
       </c>
@@ -2497,7 +2502,7 @@
       <c r="H63" s="11"/>
       <c r="I63" s="11"/>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9">
       <c r="A64" s="1">
         <v>54</v>
       </c>
@@ -2523,7 +2528,7 @@
       <c r="H64" s="11"/>
       <c r="I64" s="11"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9">
       <c r="A65" s="1">
         <v>55</v>
       </c>
@@ -2549,7 +2554,7 @@
       <c r="H65" s="11"/>
       <c r="I65" s="11"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9">
       <c r="A66" s="1">
         <v>56</v>
       </c>
@@ -2575,7 +2580,7 @@
       <c r="H66" s="11"/>
       <c r="I66" s="11"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9">
       <c r="A67" s="1">
         <v>57</v>
       </c>
@@ -2601,7 +2606,7 @@
       <c r="H67" s="11"/>
       <c r="I67" s="11"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9">
       <c r="A68" s="1">
         <v>58</v>
       </c>
@@ -2627,7 +2632,7 @@
       <c r="H68" s="11"/>
       <c r="I68" s="11"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9">
       <c r="A69" s="1">
         <v>59</v>
       </c>
@@ -2653,7 +2658,7 @@
       <c r="H69" s="11"/>
       <c r="I69" s="11"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9">
       <c r="A70" s="1">
         <v>60</v>
       </c>
@@ -2679,7 +2684,7 @@
       <c r="H70" s="11"/>
       <c r="I70" s="11"/>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9">
       <c r="A71" s="1">
         <v>61</v>
       </c>
@@ -2705,7 +2710,7 @@
       <c r="H71" s="11"/>
       <c r="I71" s="11"/>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9">
       <c r="A72" s="1">
         <v>62</v>
       </c>
@@ -2731,7 +2736,7 @@
       <c r="H72" s="11"/>
       <c r="I72" s="11"/>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9">
       <c r="A73" s="1">
         <v>63</v>
       </c>
@@ -2757,7 +2762,7 @@
       <c r="H73" s="11"/>
       <c r="I73" s="11"/>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9">
       <c r="A74" s="1">
         <v>64</v>
       </c>
@@ -2783,7 +2788,7 @@
       <c r="H74" s="11"/>
       <c r="I74" s="11"/>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9">
       <c r="A75" s="1">
         <v>65</v>
       </c>
@@ -2809,7 +2814,7 @@
       <c r="H75" s="11"/>
       <c r="I75" s="11"/>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9">
       <c r="A76" s="1">
         <v>66</v>
       </c>
@@ -2835,7 +2840,7 @@
       <c r="H76" s="11"/>
       <c r="I76" s="11"/>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9">
       <c r="A77" s="1">
         <v>67</v>
       </c>
@@ -2861,7 +2866,7 @@
       <c r="H77" s="11"/>
       <c r="I77" s="11"/>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9">
       <c r="A78" s="1">
         <v>68</v>
       </c>
@@ -2887,7 +2892,7 @@
       <c r="H78" s="11"/>
       <c r="I78" s="11"/>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9">
       <c r="A79" s="1">
         <v>69</v>
       </c>
@@ -2913,7 +2918,7 @@
       <c r="H79" s="11"/>
       <c r="I79" s="11"/>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9">
       <c r="A80" s="1">
         <v>70</v>
       </c>
@@ -2939,7 +2944,7 @@
       <c r="H80" s="11"/>
       <c r="I80" s="11"/>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9">
       <c r="A81" s="1">
         <v>71</v>
       </c>
@@ -2965,7 +2970,7 @@
       <c r="H81" s="11"/>
       <c r="I81" s="11"/>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9">
       <c r="A82" s="1">
         <v>72</v>
       </c>
@@ -2991,7 +2996,7 @@
       <c r="H82" s="11"/>
       <c r="I82" s="11"/>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9">
       <c r="A83" s="1">
         <v>73</v>
       </c>
@@ -3017,7 +3022,7 @@
       <c r="H83" s="11"/>
       <c r="I83" s="11"/>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9">
       <c r="A84" s="1">
         <v>74</v>
       </c>
@@ -3043,7 +3048,7 @@
       <c r="H84" s="11"/>
       <c r="I84" s="11"/>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9">
       <c r="A85" s="1">
         <v>75</v>
       </c>
@@ -3069,7 +3074,7 @@
       <c r="H85" s="11"/>
       <c r="I85" s="11"/>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9">
       <c r="A86" s="1">
         <v>76</v>
       </c>
@@ -3095,7 +3100,7 @@
       <c r="H86" s="11"/>
       <c r="I86" s="11"/>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9">
       <c r="A87" s="1">
         <v>77</v>
       </c>
@@ -3121,7 +3126,7 @@
       <c r="H87" s="11"/>
       <c r="I87" s="11"/>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9">
       <c r="A88" s="1">
         <v>78</v>
       </c>
@@ -3147,7 +3152,7 @@
       <c r="H88" s="11"/>
       <c r="I88" s="11"/>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9">
       <c r="A89" s="1">
         <v>79</v>
       </c>
@@ -3173,7 +3178,7 @@
       <c r="H89" s="11"/>
       <c r="I89" s="11"/>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9">
       <c r="A90" s="1">
         <v>80</v>
       </c>
@@ -3199,7 +3204,7 @@
       <c r="H90" s="11"/>
       <c r="I90" s="11"/>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9">
       <c r="A91" s="1">
         <v>81</v>
       </c>
@@ -3225,7 +3230,7 @@
       <c r="H91" s="11"/>
       <c r="I91" s="11"/>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9">
       <c r="A92" s="1">
         <v>82</v>
       </c>
@@ -3251,7 +3256,7 @@
       <c r="H92" s="11"/>
       <c r="I92" s="11"/>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9">
       <c r="A93" s="1">
         <v>83</v>
       </c>
@@ -3277,7 +3282,7 @@
       <c r="H93" s="11"/>
       <c r="I93" s="11"/>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9">
       <c r="A94" s="1">
         <v>84</v>
       </c>
@@ -3303,7 +3308,7 @@
       <c r="H94" s="11"/>
       <c r="I94" s="11"/>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9">
       <c r="A95" s="1">
         <v>85</v>
       </c>
@@ -3329,7 +3334,7 @@
       <c r="H95" s="11"/>
       <c r="I95" s="11"/>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9">
       <c r="A96" s="1">
         <v>86</v>
       </c>
@@ -3355,7 +3360,7 @@
       <c r="H96" s="11"/>
       <c r="I96" s="11"/>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9">
       <c r="A97" s="1">
         <v>87</v>
       </c>
@@ -3381,7 +3386,7 @@
       <c r="H97" s="11"/>
       <c r="I97" s="11"/>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9">
       <c r="A98" s="1">
         <v>88</v>
       </c>
@@ -3407,7 +3412,7 @@
       <c r="H98" s="11"/>
       <c r="I98" s="11"/>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9">
       <c r="A99" s="1">
         <v>89</v>
       </c>
@@ -3433,7 +3438,7 @@
       <c r="H99" s="11"/>
       <c r="I99" s="11"/>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9">
       <c r="A100" s="1">
         <v>90</v>
       </c>
@@ -3459,7 +3464,7 @@
       <c r="H100" s="11"/>
       <c r="I100" s="11"/>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9">
       <c r="A101" s="1">
         <v>91</v>
       </c>
@@ -3485,7 +3490,7 @@
       <c r="H101" s="11"/>
       <c r="I101" s="11"/>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9">
       <c r="A102" s="1">
         <v>92</v>
       </c>
@@ -3511,7 +3516,7 @@
       <c r="H102" s="11"/>
       <c r="I102" s="11"/>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9">
       <c r="A103" s="1">
         <v>93</v>
       </c>
@@ -3537,7 +3542,7 @@
       <c r="H103" s="11"/>
       <c r="I103" s="11"/>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9">
       <c r="A104" s="1">
         <v>94</v>
       </c>
@@ -3563,7 +3568,7 @@
       <c r="H104" s="11"/>
       <c r="I104" s="11"/>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9">
       <c r="A105" s="1">
         <v>95</v>
       </c>
@@ -3589,7 +3594,7 @@
       <c r="H105" s="11"/>
       <c r="I105" s="11"/>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9">
       <c r="A106" s="1">
         <v>96</v>
       </c>
@@ -3615,7 +3620,7 @@
       <c r="H106" s="11"/>
       <c r="I106" s="11"/>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9">
       <c r="A107" s="1">
         <v>97</v>
       </c>
@@ -3641,7 +3646,7 @@
       <c r="H107" s="11"/>
       <c r="I107" s="11"/>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9">
       <c r="A108" s="1">
         <v>98</v>
       </c>
@@ -3667,7 +3672,7 @@
       <c r="H108" s="11"/>
       <c r="I108" s="11"/>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9">
       <c r="A109" s="1">
         <v>99</v>
       </c>
@@ -3693,7 +3698,7 @@
       <c r="H109" s="11"/>
       <c r="I109" s="11"/>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9">
       <c r="A110" s="1">
         <v>100</v>
       </c>
@@ -3719,7 +3724,7 @@
       <c r="H110" s="11"/>
       <c r="I110" s="11"/>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9">
       <c r="A111" s="1">
         <v>101</v>
       </c>
@@ -3745,7 +3750,7 @@
       <c r="H111" s="11"/>
       <c r="I111" s="11"/>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9">
       <c r="A112" s="1">
         <v>102</v>
       </c>
@@ -3771,7 +3776,7 @@
       <c r="H112" s="11"/>
       <c r="I112" s="11"/>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9">
       <c r="A113" s="1">
         <v>103</v>
       </c>
@@ -3797,7 +3802,7 @@
       <c r="H113" s="11"/>
       <c r="I113" s="11"/>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9">
       <c r="A114" s="1">
         <v>104</v>
       </c>
@@ -3823,7 +3828,7 @@
       <c r="H114" s="11"/>
       <c r="I114" s="11"/>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9">
       <c r="A115" s="1">
         <v>105</v>
       </c>
@@ -3849,7 +3854,7 @@
       <c r="H115" s="11"/>
       <c r="I115" s="11"/>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9">
       <c r="A116" s="1">
         <v>106</v>
       </c>
@@ -3875,7 +3880,7 @@
       <c r="H116" s="11"/>
       <c r="I116" s="11"/>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9">
       <c r="A117" s="1">
         <v>107</v>
       </c>
@@ -3901,7 +3906,7 @@
       <c r="H117" s="11"/>
       <c r="I117" s="11"/>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9">
       <c r="A118" s="1">
         <v>108</v>
       </c>
@@ -3927,7 +3932,7 @@
       <c r="H118" s="11"/>
       <c r="I118" s="11"/>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9">
       <c r="A119" s="1">
         <v>109</v>
       </c>
@@ -3953,7 +3958,7 @@
       <c r="H119" s="11"/>
       <c r="I119" s="11"/>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9">
       <c r="A120" s="1">
         <v>110</v>
       </c>
@@ -3979,7 +3984,7 @@
       <c r="H120" s="11"/>
       <c r="I120" s="11"/>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9">
       <c r="A121" s="1">
         <v>111</v>
       </c>
@@ -4005,7 +4010,7 @@
       <c r="H121" s="11"/>
       <c r="I121" s="11"/>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9">
       <c r="A122" s="1">
         <v>112</v>
       </c>
@@ -4031,7 +4036,7 @@
       <c r="H122" s="11"/>
       <c r="I122" s="11"/>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9">
       <c r="A123" s="1">
         <v>113</v>
       </c>
@@ -4057,7 +4062,7 @@
       <c r="H123" s="11"/>
       <c r="I123" s="11"/>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9">
       <c r="A124" s="1">
         <v>114</v>
       </c>
@@ -4083,7 +4088,7 @@
       <c r="H124" s="11"/>
       <c r="I124" s="11"/>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9">
       <c r="A125" s="1">
         <v>115</v>
       </c>
@@ -4109,7 +4114,7 @@
       <c r="H125" s="11"/>
       <c r="I125" s="11"/>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9">
       <c r="A126" s="1">
         <v>116</v>
       </c>
@@ -4135,7 +4140,7 @@
       <c r="H126" s="11"/>
       <c r="I126" s="11"/>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9">
       <c r="A127" s="1">
         <v>117</v>
       </c>
@@ -4161,7 +4166,7 @@
       <c r="H127" s="11"/>
       <c r="I127" s="11"/>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9">
       <c r="A128" s="1">
         <v>118</v>
       </c>
@@ -4187,7 +4192,7 @@
       <c r="H128" s="11"/>
       <c r="I128" s="11"/>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9">
       <c r="A129" s="1">
         <v>119</v>
       </c>
@@ -4213,7 +4218,7 @@
       <c r="H129" s="11"/>
       <c r="I129" s="11"/>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:9">
       <c r="A130" s="1">
         <v>120</v>
       </c>
@@ -4239,7 +4244,7 @@
       <c r="H130" s="11"/>
       <c r="I130" s="11"/>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:9">
       <c r="A131" s="1">
         <v>121</v>
       </c>
@@ -4265,7 +4270,7 @@
       <c r="H131" s="11"/>
       <c r="I131" s="11"/>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9">
       <c r="A132" s="1">
         <v>122</v>
       </c>
@@ -4291,7 +4296,7 @@
       <c r="H132" s="11"/>
       <c r="I132" s="11"/>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9">
       <c r="A133" s="1">
         <v>123</v>
       </c>
@@ -4317,7 +4322,7 @@
       <c r="H133" s="11"/>
       <c r="I133" s="11"/>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9">
       <c r="A134" s="1">
         <v>124</v>
       </c>
@@ -4343,7 +4348,7 @@
       <c r="H134" s="11"/>
       <c r="I134" s="11"/>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:9">
       <c r="A135" s="1">
         <v>125</v>
       </c>
@@ -4369,7 +4374,7 @@
       <c r="H135" s="11"/>
       <c r="I135" s="11"/>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:9">
       <c r="A136" s="1">
         <v>126</v>
       </c>
@@ -4395,7 +4400,7 @@
       <c r="H136" s="11"/>
       <c r="I136" s="11"/>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:9">
       <c r="A137" s="1">
         <v>127</v>
       </c>
@@ -4421,7 +4426,7 @@
       <c r="H137" s="11"/>
       <c r="I137" s="11"/>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:9">
       <c r="A138" s="1">
         <v>128</v>
       </c>
@@ -4447,7 +4452,7 @@
       <c r="H138" s="11"/>
       <c r="I138" s="11"/>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:9">
       <c r="A139" s="1">
         <v>129</v>
       </c>
@@ -4473,7 +4478,7 @@
       <c r="H139" s="11"/>
       <c r="I139" s="11"/>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9">
       <c r="A140" s="1">
         <v>130</v>
       </c>
@@ -4499,7 +4504,7 @@
       <c r="H140" s="11"/>
       <c r="I140" s="11"/>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:9">
       <c r="A141" s="1">
         <v>131</v>
       </c>
@@ -4525,7 +4530,7 @@
       <c r="H141" s="11"/>
       <c r="I141" s="11"/>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:9">
       <c r="A142" s="1">
         <v>132</v>
       </c>
@@ -4551,7 +4556,7 @@
       <c r="H142" s="11"/>
       <c r="I142" s="11"/>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:9">
       <c r="A143" s="1">
         <v>133</v>
       </c>
@@ -4577,7 +4582,7 @@
       <c r="H143" s="11"/>
       <c r="I143" s="11"/>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9">
       <c r="A144" s="1">
         <v>134</v>
       </c>
@@ -4603,7 +4608,7 @@
       <c r="H144" s="11"/>
       <c r="I144" s="11"/>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9">
       <c r="A145" s="1">
         <v>135</v>
       </c>
@@ -4629,7 +4634,7 @@
       <c r="H145" s="11"/>
       <c r="I145" s="11"/>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:9">
       <c r="A146" s="1">
         <v>136</v>
       </c>
@@ -4655,7 +4660,7 @@
       <c r="H146" s="11"/>
       <c r="I146" s="11"/>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9">
       <c r="A147" s="1">
         <v>137</v>
       </c>
@@ -4681,7 +4686,7 @@
       <c r="H147" s="11"/>
       <c r="I147" s="11"/>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9">
       <c r="A148" s="1">
         <v>138</v>
       </c>
@@ -4707,7 +4712,7 @@
       <c r="H148" s="11"/>
       <c r="I148" s="11"/>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9">
       <c r="A149" s="1">
         <v>139</v>
       </c>
@@ -4733,7 +4738,7 @@
       <c r="H149" s="11"/>
       <c r="I149" s="11"/>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9">
       <c r="A150" s="1">
         <v>140</v>
       </c>
@@ -4759,7 +4764,7 @@
       <c r="H150" s="11"/>
       <c r="I150" s="11"/>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9">
       <c r="A151" s="1">
         <v>141</v>
       </c>
@@ -4785,7 +4790,7 @@
       <c r="H151" s="11"/>
       <c r="I151" s="11"/>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9">
       <c r="A152" s="1">
         <v>142</v>
       </c>
@@ -4811,7 +4816,7 @@
       <c r="H152" s="11"/>
       <c r="I152" s="11"/>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9">
       <c r="A153" s="1">
         <v>143</v>
       </c>
@@ -4837,7 +4842,7 @@
       <c r="H153" s="11"/>
       <c r="I153" s="11"/>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9">
       <c r="A154" s="1">
         <v>144</v>
       </c>
@@ -4863,7 +4868,7 @@
       <c r="H154" s="11"/>
       <c r="I154" s="11"/>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:9">
       <c r="A155" s="1">
         <v>145</v>
       </c>
@@ -4889,7 +4894,7 @@
       <c r="H155" s="11"/>
       <c r="I155" s="11"/>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:9">
       <c r="A156" s="1">
         <v>146</v>
       </c>
@@ -4915,7 +4920,7 @@
       <c r="H156" s="11"/>
       <c r="I156" s="11"/>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9">
       <c r="A157" s="1">
         <v>147</v>
       </c>
@@ -4941,7 +4946,7 @@
       <c r="H157" s="11"/>
       <c r="I157" s="11"/>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9">
       <c r="A158" s="1">
         <v>148</v>
       </c>
@@ -4967,7 +4972,7 @@
       <c r="H158" s="11"/>
       <c r="I158" s="11"/>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9">
       <c r="A159" s="1">
         <v>149</v>
       </c>
@@ -4993,7 +4998,7 @@
       <c r="H159" s="11"/>
       <c r="I159" s="11"/>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9">
       <c r="A160" s="1">
         <v>150</v>
       </c>
@@ -5019,7 +5024,7 @@
       <c r="H160" s="11"/>
       <c r="I160" s="11"/>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9">
       <c r="A161" s="1">
         <v>151</v>
       </c>
@@ -5045,7 +5050,7 @@
       <c r="H161" s="11"/>
       <c r="I161" s="11"/>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:9">
       <c r="A162" s="1">
         <v>152</v>
       </c>
@@ -5071,7 +5076,7 @@
       <c r="H162" s="11"/>
       <c r="I162" s="11"/>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:9">
       <c r="A163" s="1">
         <v>153</v>
       </c>
@@ -5097,7 +5102,7 @@
       <c r="H163" s="11"/>
       <c r="I163" s="11"/>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:9">
       <c r="A164" s="1">
         <v>154</v>
       </c>
@@ -5123,7 +5128,7 @@
       <c r="H164" s="11"/>
       <c r="I164" s="11"/>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:9">
       <c r="A165" s="1">
         <v>155</v>
       </c>
@@ -5149,7 +5154,7 @@
       <c r="H165" s="11"/>
       <c r="I165" s="11"/>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:9">
       <c r="A166" s="1">
         <v>156</v>
       </c>
@@ -5175,7 +5180,7 @@
       <c r="H166" s="11"/>
       <c r="I166" s="11"/>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:9">
       <c r="A167" s="1">
         <v>157</v>
       </c>
@@ -5201,7 +5206,7 @@
       <c r="H167" s="11"/>
       <c r="I167" s="11"/>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:9">
       <c r="A168" s="1">
         <v>158</v>
       </c>
@@ -5227,7 +5232,7 @@
       <c r="H168" s="11"/>
       <c r="I168" s="11"/>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:9">
       <c r="A169" s="1">
         <v>159</v>
       </c>
@@ -5253,7 +5258,7 @@
       <c r="H169" s="11"/>
       <c r="I169" s="11"/>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:9">
       <c r="A170" s="1">
         <v>160</v>
       </c>
@@ -5279,7 +5284,7 @@
       <c r="H170" s="11"/>
       <c r="I170" s="11"/>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:9">
       <c r="A171" s="1">
         <v>161</v>
       </c>
@@ -5305,7 +5310,7 @@
       <c r="H171" s="11"/>
       <c r="I171" s="11"/>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:9">
       <c r="A172" s="1">
         <v>162</v>
       </c>
@@ -5331,7 +5336,7 @@
       <c r="H172" s="11"/>
       <c r="I172" s="11"/>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:9">
       <c r="A173" s="1">
         <v>163</v>
       </c>
@@ -5357,7 +5362,7 @@
       <c r="H173" s="11"/>
       <c r="I173" s="11"/>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:9">
       <c r="A174" s="1">
         <v>164</v>
       </c>
@@ -5383,7 +5388,7 @@
       <c r="H174" s="11"/>
       <c r="I174" s="11"/>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:9">
       <c r="A175" s="1">
         <v>165</v>
       </c>
@@ -5409,7 +5414,7 @@
       <c r="H175" s="11"/>
       <c r="I175" s="11"/>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:9">
       <c r="A176" s="1">
         <v>166</v>
       </c>
@@ -5435,7 +5440,7 @@
       <c r="H176" s="11"/>
       <c r="I176" s="11"/>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:9">
       <c r="A177" s="1">
         <v>167</v>
       </c>
@@ -5461,7 +5466,7 @@
       <c r="H177" s="11"/>
       <c r="I177" s="11"/>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:9">
       <c r="A178" s="1">
         <v>168</v>
       </c>
@@ -5487,7 +5492,7 @@
       <c r="H178" s="11"/>
       <c r="I178" s="11"/>
     </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9">
       <c r="A179" s="1">
         <v>169</v>
       </c>
@@ -5513,7 +5518,7 @@
       <c r="H179" s="11"/>
       <c r="I179" s="11"/>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:9">
       <c r="A180" s="1">
         <v>170</v>
       </c>
@@ -5539,7 +5544,7 @@
       <c r="H180" s="11"/>
       <c r="I180" s="11"/>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:9">
       <c r="A181" s="1">
         <v>171</v>
       </c>
@@ -5565,7 +5570,7 @@
       <c r="H181" s="11"/>
       <c r="I181" s="11"/>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:9">
       <c r="A182" s="1">
         <v>172</v>
       </c>
@@ -5591,7 +5596,7 @@
       <c r="H182" s="11"/>
       <c r="I182" s="11"/>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:9">
       <c r="A183" s="1">
         <v>173</v>
       </c>
@@ -5617,7 +5622,7 @@
       <c r="H183" s="11"/>
       <c r="I183" s="11"/>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:9">
       <c r="A184" s="1">
         <v>174</v>
       </c>
@@ -5643,7 +5648,7 @@
       <c r="H184" s="11"/>
       <c r="I184" s="11"/>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:9">
       <c r="A185" s="1">
         <v>175</v>
       </c>
@@ -5669,7 +5674,7 @@
       <c r="H185" s="11"/>
       <c r="I185" s="11"/>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:9">
       <c r="A186" s="1">
         <v>176</v>
       </c>
@@ -5695,7 +5700,7 @@
       <c r="H186" s="11"/>
       <c r="I186" s="11"/>
     </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:9">
       <c r="A187" s="1">
         <v>177</v>
       </c>
@@ -5721,7 +5726,7 @@
       <c r="H187" s="11"/>
       <c r="I187" s="11"/>
     </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:9">
       <c r="A188" s="1">
         <v>178</v>
       </c>
@@ -5747,7 +5752,7 @@
       <c r="H188" s="11"/>
       <c r="I188" s="11"/>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:9">
       <c r="A189" s="1">
         <v>179</v>
       </c>
@@ -5773,7 +5778,7 @@
       <c r="H189" s="11"/>
       <c r="I189" s="11"/>
     </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:9">
       <c r="A190" s="1">
         <v>180</v>
       </c>
@@ -5799,7 +5804,7 @@
       <c r="H190" s="11"/>
       <c r="I190" s="11"/>
     </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:9">
       <c r="A191" s="1">
         <v>181</v>
       </c>
@@ -5825,7 +5830,7 @@
       <c r="H191" s="11"/>
       <c r="I191" s="11"/>
     </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:9">
       <c r="A192" s="1">
         <v>182</v>
       </c>
@@ -5851,7 +5856,7 @@
       <c r="H192" s="11"/>
       <c r="I192" s="11"/>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:9">
       <c r="A193" s="1">
         <v>183</v>
       </c>
@@ -5877,7 +5882,7 @@
       <c r="H193" s="11"/>
       <c r="I193" s="11"/>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:9">
       <c r="A194" s="1">
         <v>184</v>
       </c>
@@ -5903,7 +5908,7 @@
       <c r="H194" s="11"/>
       <c r="I194" s="11"/>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:9">
       <c r="A195" s="1">
         <v>185</v>
       </c>
@@ -5929,7 +5934,7 @@
       <c r="H195" s="11"/>
       <c r="I195" s="11"/>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:9">
       <c r="A196" s="1">
         <v>186</v>
       </c>
@@ -5955,7 +5960,7 @@
       <c r="H196" s="11"/>
       <c r="I196" s="11"/>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:9">
       <c r="A197" s="1">
         <v>187</v>
       </c>
@@ -5981,7 +5986,7 @@
       <c r="H197" s="11"/>
       <c r="I197" s="11"/>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:9">
       <c r="A198" s="1">
         <v>188</v>
       </c>
@@ -6007,7 +6012,7 @@
       <c r="H198" s="11"/>
       <c r="I198" s="11"/>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:9">
       <c r="A199" s="1">
         <v>189</v>
       </c>
@@ -6033,7 +6038,7 @@
       <c r="H199" s="11"/>
       <c r="I199" s="11"/>
     </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:9">
       <c r="A200" s="1">
         <v>190</v>
       </c>
@@ -6059,7 +6064,7 @@
       <c r="H200" s="11"/>
       <c r="I200" s="11"/>
     </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:9">
       <c r="A201" s="1">
         <v>191</v>
       </c>
@@ -6085,7 +6090,7 @@
       <c r="H201" s="11"/>
       <c r="I201" s="11"/>
     </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:9">
       <c r="A202" s="1">
         <v>192</v>
       </c>
@@ -6111,7 +6116,7 @@
       <c r="H202" s="11"/>
       <c r="I202" s="11"/>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:9">
       <c r="A203" s="1">
         <v>193</v>
       </c>
@@ -6137,7 +6142,7 @@
       <c r="H203" s="11"/>
       <c r="I203" s="11"/>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9">
       <c r="A204" s="1">
         <v>194</v>
       </c>
@@ -6163,7 +6168,7 @@
       <c r="H204" s="11"/>
       <c r="I204" s="11"/>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9">
       <c r="A205" s="1">
         <v>195</v>
       </c>
@@ -6189,7 +6194,7 @@
       <c r="H205" s="11"/>
       <c r="I205" s="11"/>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:9">
       <c r="A206" s="1">
         <v>196</v>
       </c>
@@ -6215,7 +6220,7 @@
       <c r="H206" s="11"/>
       <c r="I206" s="11"/>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:9">
       <c r="A207" s="1">
         <v>197</v>
       </c>
@@ -6241,7 +6246,7 @@
       <c r="H207" s="11"/>
       <c r="I207" s="11"/>
     </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:9">
       <c r="A208" s="1">
         <v>198</v>
       </c>
@@ -6267,7 +6272,7 @@
       <c r="H208" s="11"/>
       <c r="I208" s="11"/>
     </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:9">
       <c r="A209" s="1">
         <v>199</v>
       </c>
@@ -6293,7 +6298,7 @@
       <c r="H209" s="11"/>
       <c r="I209" s="11"/>
     </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:9">
       <c r="A210" s="1">
         <v>200</v>
       </c>
@@ -6319,7 +6324,7 @@
       <c r="H210" s="11"/>
       <c r="I210" s="11"/>
     </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:9">
       <c r="A211" s="1">
         <v>201</v>
       </c>
@@ -6345,7 +6350,7 @@
       <c r="H211" s="11"/>
       <c r="I211" s="11"/>
     </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:9">
       <c r="A212" s="1">
         <v>202</v>
       </c>
@@ -6371,7 +6376,7 @@
       <c r="H212" s="11"/>
       <c r="I212" s="11"/>
     </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:9">
       <c r="A213" s="1">
         <v>203</v>
       </c>
@@ -6397,7 +6402,7 @@
       <c r="H213" s="11"/>
       <c r="I213" s="11"/>
     </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:9">
       <c r="A214" s="1">
         <v>204</v>
       </c>
@@ -6423,7 +6428,7 @@
       <c r="H214" s="11"/>
       <c r="I214" s="11"/>
     </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:9">
       <c r="A215" s="1">
         <v>205</v>
       </c>
@@ -6449,7 +6454,7 @@
       <c r="H215" s="11"/>
       <c r="I215" s="11"/>
     </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:9">
       <c r="A216" s="1">
         <v>206</v>
       </c>
@@ -6475,7 +6480,7 @@
       <c r="H216" s="11"/>
       <c r="I216" s="11"/>
     </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:9">
       <c r="A217" s="1">
         <v>207</v>
       </c>
@@ -6501,7 +6506,7 @@
       <c r="H217" s="11"/>
       <c r="I217" s="11"/>
     </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:9">
       <c r="A218" s="1">
         <v>208</v>
       </c>
@@ -6527,7 +6532,7 @@
       <c r="H218" s="11"/>
       <c r="I218" s="11"/>
     </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:9">
       <c r="A219" s="1">
         <v>209</v>
       </c>
@@ -6553,7 +6558,7 @@
       <c r="H219" s="11"/>
       <c r="I219" s="11"/>
     </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:9">
       <c r="A220" s="1">
         <v>210</v>
       </c>
@@ -6579,7 +6584,7 @@
       <c r="H220" s="11"/>
       <c r="I220" s="11"/>
     </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:9">
       <c r="A221" s="1">
         <v>211</v>
       </c>
@@ -6605,7 +6610,7 @@
       <c r="H221" s="11"/>
       <c r="I221" s="11"/>
     </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:9">
       <c r="A222" s="1">
         <v>212</v>
       </c>
@@ -6631,7 +6636,7 @@
       <c r="H222" s="11"/>
       <c r="I222" s="11"/>
     </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:9">
       <c r="A223" s="1">
         <v>213</v>
       </c>
@@ -6657,7 +6662,7 @@
       <c r="H223" s="11"/>
       <c r="I223" s="11"/>
     </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:9">
       <c r="A224" s="1">
         <v>214</v>
       </c>
@@ -6683,7 +6688,7 @@
       <c r="H224" s="11"/>
       <c r="I224" s="11"/>
     </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:9">
       <c r="A225" s="1">
         <v>215</v>
       </c>
@@ -6709,7 +6714,7 @@
       <c r="H225" s="11"/>
       <c r="I225" s="11"/>
     </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:9">
       <c r="A226" s="1">
         <v>216</v>
       </c>
@@ -6735,7 +6740,7 @@
       <c r="H226" s="11"/>
       <c r="I226" s="11"/>
     </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:9">
       <c r="A227" s="1">
         <v>217</v>
       </c>
@@ -6761,7 +6766,7 @@
       <c r="H227" s="11"/>
       <c r="I227" s="11"/>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:9">
       <c r="A228" s="1">
         <v>218</v>
       </c>
@@ -6787,7 +6792,7 @@
       <c r="H228" s="11"/>
       <c r="I228" s="11"/>
     </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:9">
       <c r="A229" s="1">
         <v>219</v>
       </c>
@@ -6813,7 +6818,7 @@
       <c r="H229" s="11"/>
       <c r="I229" s="11"/>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:9">
       <c r="A230" s="1">
         <v>220</v>
       </c>
@@ -6839,7 +6844,7 @@
       <c r="H230" s="11"/>
       <c r="I230" s="11"/>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:9">
       <c r="A231" s="1">
         <v>221</v>
       </c>
@@ -6865,7 +6870,7 @@
       <c r="H231" s="11"/>
       <c r="I231" s="11"/>
     </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:9">
       <c r="A232" s="1">
         <v>222</v>
       </c>
@@ -6891,7 +6896,7 @@
       <c r="H232" s="11"/>
       <c r="I232" s="11"/>
     </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:9">
       <c r="A233" s="1">
         <v>223</v>
       </c>
@@ -6917,7 +6922,7 @@
       <c r="H233" s="11"/>
       <c r="I233" s="11"/>
     </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:9">
       <c r="A234" s="1">
         <v>224</v>
       </c>
@@ -6943,7 +6948,7 @@
       <c r="H234" s="11"/>
       <c r="I234" s="11"/>
     </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:9">
       <c r="A235" s="1">
         <v>225</v>
       </c>
@@ -6969,7 +6974,7 @@
       <c r="H235" s="11"/>
       <c r="I235" s="11"/>
     </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:9">
       <c r="A236" s="1">
         <v>226</v>
       </c>
@@ -6995,7 +7000,7 @@
       <c r="H236" s="11"/>
       <c r="I236" s="11"/>
     </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:9">
       <c r="A237" s="1">
         <v>227</v>
       </c>
@@ -7021,7 +7026,7 @@
       <c r="H237" s="11"/>
       <c r="I237" s="11"/>
     </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:9">
       <c r="A238" s="1">
         <v>228</v>
       </c>
@@ -7047,7 +7052,7 @@
       <c r="H238" s="11"/>
       <c r="I238" s="11"/>
     </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:9">
       <c r="A239" s="1">
         <v>229</v>
       </c>
@@ -7073,7 +7078,7 @@
       <c r="H239" s="11"/>
       <c r="I239" s="11"/>
     </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:9">
       <c r="A240" s="1">
         <v>230</v>
       </c>
@@ -7099,7 +7104,7 @@
       <c r="H240" s="11"/>
       <c r="I240" s="11"/>
     </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:9">
       <c r="A241" s="1">
         <v>231</v>
       </c>
@@ -7125,7 +7130,7 @@
       <c r="H241" s="11"/>
       <c r="I241" s="11"/>
     </row>
-    <row r="242" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:9">
       <c r="A242" s="1">
         <v>232</v>
       </c>
@@ -7151,7 +7156,7 @@
       <c r="H242" s="11"/>
       <c r="I242" s="11"/>
     </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:9">
       <c r="A243" s="1">
         <v>233</v>
       </c>
@@ -7177,7 +7182,7 @@
       <c r="H243" s="11"/>
       <c r="I243" s="11"/>
     </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:9">
       <c r="A244" s="1">
         <v>234</v>
       </c>
@@ -7203,7 +7208,7 @@
       <c r="H244" s="11"/>
       <c r="I244" s="11"/>
     </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:9">
       <c r="A245" s="1">
         <v>235</v>
       </c>
@@ -7229,7 +7234,7 @@
       <c r="H245" s="11"/>
       <c r="I245" s="11"/>
     </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:9">
       <c r="A246" s="1">
         <v>236</v>
       </c>
@@ -7255,7 +7260,7 @@
       <c r="H246" s="11"/>
       <c r="I246" s="11"/>
     </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:9">
       <c r="A247" s="1">
         <v>237</v>
       </c>
@@ -7281,7 +7286,7 @@
       <c r="H247" s="11"/>
       <c r="I247" s="11"/>
     </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:9">
       <c r="A248" s="1">
         <v>238</v>
       </c>
@@ -7307,7 +7312,7 @@
       <c r="H248" s="11"/>
       <c r="I248" s="11"/>
     </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:9">
       <c r="A249" s="1">
         <v>239</v>
       </c>
@@ -7333,7 +7338,7 @@
       <c r="H249" s="11"/>
       <c r="I249" s="11"/>
     </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:9">
       <c r="A250" s="1">
         <v>240</v>
       </c>
@@ -7359,7 +7364,7 @@
       <c r="H250" s="11"/>
       <c r="I250" s="11"/>
     </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:9">
       <c r="A251" s="1">
         <v>241</v>
       </c>
@@ -7385,7 +7390,7 @@
       <c r="H251" s="11"/>
       <c r="I251" s="11"/>
     </row>
-    <row r="252" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:9">
       <c r="A252" s="1">
         <v>242</v>
       </c>
@@ -7411,7 +7416,7 @@
       <c r="H252" s="11"/>
       <c r="I252" s="11"/>
     </row>
-    <row r="253" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:9">
       <c r="A253" s="1">
         <v>243</v>
       </c>
@@ -7437,7 +7442,7 @@
       <c r="H253" s="11"/>
       <c r="I253" s="11"/>
     </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:9">
       <c r="A254" s="1">
         <v>244</v>
       </c>
@@ -7463,7 +7468,7 @@
       <c r="H254" s="11"/>
       <c r="I254" s="11"/>
     </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:9">
       <c r="A255" s="1">
         <v>245</v>
       </c>
@@ -7489,7 +7494,7 @@
       <c r="H255" s="11"/>
       <c r="I255" s="11"/>
     </row>
-    <row r="256" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:9">
       <c r="A256" s="1">
         <v>246</v>
       </c>
@@ -7515,7 +7520,7 @@
       <c r="H256" s="11"/>
       <c r="I256" s="11"/>
     </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:9">
       <c r="A257" s="1">
         <v>247</v>
       </c>
@@ -7541,7 +7546,7 @@
       <c r="H257" s="11"/>
       <c r="I257" s="11"/>
     </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:9">
       <c r="A258" s="1">
         <v>248</v>
       </c>
@@ -7567,7 +7572,7 @@
       <c r="H258" s="11"/>
       <c r="I258" s="11"/>
     </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:9">
       <c r="A259" s="1">
         <v>249</v>
       </c>
@@ -7593,7 +7598,7 @@
       <c r="H259" s="11"/>
       <c r="I259" s="11"/>
     </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:9">
       <c r="A260" s="1">
         <v>250</v>
       </c>
@@ -7619,7 +7624,7 @@
       <c r="H260" s="11"/>
       <c r="I260" s="11"/>
     </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:9">
       <c r="A261" s="1">
         <v>251</v>
       </c>
@@ -7645,7 +7650,7 @@
       <c r="H261" s="11"/>
       <c r="I261" s="11"/>
     </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:9">
       <c r="A262" s="1">
         <v>252</v>
       </c>
@@ -7671,7 +7676,7 @@
       <c r="H262" s="11"/>
       <c r="I262" s="11"/>
     </row>
-    <row r="263" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:9">
       <c r="A263" s="1">
         <v>253</v>
       </c>
@@ -7697,7 +7702,7 @@
       <c r="H263" s="11"/>
       <c r="I263" s="11"/>
     </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:9">
       <c r="A264" s="1">
         <v>254</v>
       </c>
@@ -7723,7 +7728,7 @@
       <c r="H264" s="11"/>
       <c r="I264" s="11"/>
     </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:9">
       <c r="A265" s="1">
         <v>255</v>
       </c>
@@ -7749,7 +7754,7 @@
       <c r="H265" s="11"/>
       <c r="I265" s="11"/>
     </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:9">
       <c r="A266" s="1">
         <v>256</v>
       </c>
@@ -7775,7 +7780,7 @@
       <c r="H266" s="11"/>
       <c r="I266" s="11"/>
     </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:9">
       <c r="A267" s="1">
         <v>257</v>
       </c>
@@ -7801,7 +7806,7 @@
       <c r="H267" s="11"/>
       <c r="I267" s="11"/>
     </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:9">
       <c r="A268" s="1">
         <v>258</v>
       </c>
@@ -7827,7 +7832,7 @@
       <c r="H268" s="11"/>
       <c r="I268" s="11"/>
     </row>
-    <row r="269" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:9">
       <c r="A269" s="1">
         <v>259</v>
       </c>
@@ -7853,7 +7858,7 @@
       <c r="H269" s="11"/>
       <c r="I269" s="11"/>
     </row>
-    <row r="270" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:9">
       <c r="A270" s="1">
         <v>260</v>
       </c>
@@ -7879,7 +7884,7 @@
       <c r="H270" s="11"/>
       <c r="I270" s="11"/>
     </row>
-    <row r="271" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:9">
       <c r="A271" s="1">
         <v>261</v>
       </c>
@@ -7905,7 +7910,7 @@
       <c r="H271" s="11"/>
       <c r="I271" s="11"/>
     </row>
-    <row r="272" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:9">
       <c r="A272" s="1">
         <v>262</v>
       </c>
@@ -7931,7 +7936,7 @@
       <c r="H272" s="11"/>
       <c r="I272" s="11"/>
     </row>
-    <row r="273" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:9">
       <c r="A273" s="1">
         <v>263</v>
       </c>
@@ -7957,7 +7962,7 @@
       <c r="H273" s="11"/>
       <c r="I273" s="11"/>
     </row>
-    <row r="274" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:9">
       <c r="A274" s="1">
         <v>264</v>
       </c>
@@ -7983,7 +7988,7 @@
       <c r="H274" s="11"/>
       <c r="I274" s="11"/>
     </row>
-    <row r="275" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:9">
       <c r="A275" s="1">
         <v>265</v>
       </c>
@@ -8009,7 +8014,7 @@
       <c r="H275" s="11"/>
       <c r="I275" s="11"/>
     </row>
-    <row r="276" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:9">
       <c r="A276" s="1">
         <v>266</v>
       </c>
@@ -8035,7 +8040,7 @@
       <c r="H276" s="11"/>
       <c r="I276" s="11"/>
     </row>
-    <row r="277" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:9">
       <c r="A277" s="1">
         <v>267</v>
       </c>
@@ -8061,7 +8066,7 @@
       <c r="H277" s="11"/>
       <c r="I277" s="11"/>
     </row>
-    <row r="278" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:9">
       <c r="A278" s="1">
         <v>268</v>
       </c>
@@ -8087,7 +8092,7 @@
       <c r="H278" s="11"/>
       <c r="I278" s="11"/>
     </row>
-    <row r="279" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:9">
       <c r="A279" s="1">
         <v>269</v>
       </c>
@@ -8113,7 +8118,7 @@
       <c r="H279" s="11"/>
       <c r="I279" s="11"/>
     </row>
-    <row r="280" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:9">
       <c r="A280" s="1">
         <v>270</v>
       </c>
@@ -8139,7 +8144,7 @@
       <c r="H280" s="11"/>
       <c r="I280" s="11"/>
     </row>
-    <row r="281" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:9">
       <c r="A281" s="1">
         <v>271</v>
       </c>
@@ -8165,7 +8170,7 @@
       <c r="H281" s="11"/>
       <c r="I281" s="11"/>
     </row>
-    <row r="282" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:9">
       <c r="A282" s="1">
         <v>272</v>
       </c>
@@ -8191,7 +8196,7 @@
       <c r="H282" s="11"/>
       <c r="I282" s="11"/>
     </row>
-    <row r="283" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:9">
       <c r="A283" s="1">
         <v>273</v>
       </c>
@@ -8217,7 +8222,7 @@
       <c r="H283" s="11"/>
       <c r="I283" s="11"/>
     </row>
-    <row r="284" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:9">
       <c r="A284" s="1">
         <v>274</v>
       </c>
@@ -8243,7 +8248,7 @@
       <c r="H284" s="11"/>
       <c r="I284" s="11"/>
     </row>
-    <row r="285" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:9">
       <c r="A285" s="1">
         <v>275</v>
       </c>
@@ -8269,7 +8274,7 @@
       <c r="H285" s="11"/>
       <c r="I285" s="11"/>
     </row>
-    <row r="286" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:9">
       <c r="A286" s="1">
         <v>276</v>
       </c>
@@ -8299,7 +8304,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="287" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:9">
       <c r="A287" s="1">
         <v>277</v>
       </c>
@@ -8329,7 +8334,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="288" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:9">
       <c r="A288" s="1">
         <v>278</v>
       </c>
@@ -8359,7 +8364,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="289" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:9">
       <c r="A289" s="1">
         <v>279</v>
       </c>
@@ -8389,7 +8394,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="290" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:9">
       <c r="A290" s="1">
         <v>280</v>
       </c>
@@ -8419,7 +8424,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="291" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:9">
       <c r="A291" s="1">
         <v>281</v>
       </c>
@@ -8449,7 +8454,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="292" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:9">
       <c r="A292" s="1">
         <v>282</v>
       </c>
@@ -8479,7 +8484,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="293" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:9">
       <c r="A293" s="1">
         <v>283</v>
       </c>
@@ -8509,7 +8514,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="294" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:9">
       <c r="A294" s="1">
         <v>284</v>
       </c>
@@ -8539,7 +8544,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="295" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:9">
       <c r="A295" s="1">
         <v>285</v>
       </c>
@@ -8569,7 +8574,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="296" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:9">
       <c r="A296" s="1">
         <v>286</v>
       </c>
@@ -8599,7 +8604,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="297" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:9">
       <c r="A297" s="1">
         <v>287</v>
       </c>
@@ -8629,7 +8634,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="298" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:9">
       <c r="A298" s="1">
         <v>288</v>
       </c>
@@ -8659,7 +8664,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="299" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:9">
       <c r="A299" s="1">
         <v>289</v>
       </c>
@@ -8689,7 +8694,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="300" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:9">
       <c r="A300" s="1">
         <v>290</v>
       </c>
@@ -8719,7 +8724,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="301" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:9">
       <c r="A301" s="1">
         <v>291</v>
       </c>
@@ -8749,7 +8754,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="302" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:9">
       <c r="A302" s="1">
         <v>292</v>
       </c>
@@ -8779,7 +8784,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="303" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:9" s="1" customFormat="1">
       <c r="A303" s="1">
         <v>293</v>
       </c>
@@ -8809,7 +8814,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="304" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:9" s="1" customFormat="1">
       <c r="A304" s="1">
         <v>294</v>
       </c>
@@ -8839,7 +8844,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="305" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:9">
       <c r="A305" s="1">
         <v>295</v>
       </c>
@@ -8869,7 +8874,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="306" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:9">
       <c r="A306" s="1">
         <v>296</v>
       </c>
@@ -8899,7 +8904,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="307" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:9">
       <c r="A307" s="1">
         <v>297</v>
       </c>
@@ -8929,7 +8934,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="308" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:9">
       <c r="A308" s="1">
         <v>298</v>
       </c>
@@ -8959,73 +8964,73 @@
         <v>56</v>
       </c>
     </row>
-    <row r="309" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:9">
       <c r="A309" s="1"/>
     </row>
-    <row r="310" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:9">
       <c r="A310" s="1"/>
     </row>
-    <row r="311" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:9">
       <c r="A311" s="1"/>
     </row>
-    <row r="312" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:9">
       <c r="A312" s="1"/>
     </row>
-    <row r="313" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:9">
       <c r="A313" s="1"/>
     </row>
-    <row r="314" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:9">
       <c r="A314" s="1"/>
     </row>
-    <row r="315" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:9">
       <c r="A315" s="1"/>
     </row>
-    <row r="316" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:9">
       <c r="A316" s="1"/>
     </row>
-    <row r="317" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:9">
       <c r="A317" s="1"/>
     </row>
-    <row r="318" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:9">
       <c r="A318" s="1"/>
     </row>
-    <row r="319" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:9">
       <c r="A319" s="1"/>
     </row>
-    <row r="320" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:9">
       <c r="A320" s="1"/>
     </row>
-    <row r="321" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:1">
       <c r="A321" s="1"/>
     </row>
-    <row r="322" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:1">
       <c r="A322" s="1"/>
     </row>
-    <row r="323" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:1">
       <c r="A323" s="1"/>
     </row>
-    <row r="324" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:1">
       <c r="A324" s="1"/>
     </row>
-    <row r="325" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:1">
       <c r="A325" s="1"/>
     </row>
-    <row r="326" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:1">
       <c r="A326" s="1"/>
     </row>
-    <row r="327" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:1">
       <c r="A327" s="1"/>
     </row>
-    <row r="328" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:1">
       <c r="A328" s="1"/>
     </row>
-    <row r="329" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:1">
       <c r="A329" s="1"/>
     </row>
-    <row r="330" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:1">
       <c r="A330" s="1"/>
     </row>
-    <row r="331" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:1">
       <c r="A331" s="1"/>
     </row>
   </sheetData>
@@ -9047,13 +9052,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{797F1036-D41E-43A4-9E6E-CBBB62F3CD31}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="13.28515625" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -9067,7 +9072,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -9081,7 +9086,7 @@
         <v>234.67</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -9095,7 +9100,7 @@
         <v>161.15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -9109,7 +9114,7 @@
         <v>157.61000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -9123,7 +9128,7 @@
         <v>347.95</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -9137,7 +9142,7 @@
         <v>393.57</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -9151,7 +9156,7 @@
         <v>19.87</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -9165,7 +9170,7 @@
         <v>19.57</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -9179,7 +9184,7 @@
         <v>19.86</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -9193,7 +9198,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -9218,7 +9223,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56220E0F-EC16-4A8C-9E04-C7F8849C4B4D}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -9226,7 +9231,7 @@
     <col min="5" max="5" width="30.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -9243,7 +9248,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -9260,7 +9265,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -9277,7 +9282,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -9294,7 +9299,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -9311,7 +9316,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -9328,7 +9333,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -9345,7 +9350,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -9373,14 +9378,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83DAFC4B-C207-418A-8501-0E1EC9E673B7}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -9391,7 +9396,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -9402,7 +9407,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -9413,7 +9418,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -9424,7 +9429,7 @@
         <v>46517</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>61</v>
       </c>
@@ -9435,7 +9440,7 @@
         <v>46517</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -9446,7 +9451,7 @@
         <v>46631</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -9457,7 +9462,7 @@
         <v>48579</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -9468,7 +9473,7 @@
         <v>46517</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -9479,7 +9484,7 @@
         <v>46517</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -9490,7 +9495,7 @@
         <v>48579</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -9510,6 +9515,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="33ab045e-9213-4eea-a9f2-a5b809105d1e">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -9518,7 +9537,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100FB7AAE8C8816FD47B559A0CCF555AFF0" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5c9910934a78ddf693a6b708b52e9b37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f95d585e-e7a7-414c-955d-38a47c8579bd" xmlns:ns3="33ab045e-9213-4eea-a9f2-a5b809105d1e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a9c61c95b4e11caed4e46447c2ca01e7" ns2:_="" ns3:_="">
     <xsd:import namespace="f95d585e-e7a7-414c-955d-38a47c8579bd"/>
@@ -9721,47 +9740,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="33ab045e-9213-4eea-a9f2-a5b809105d1e">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59A15667-1AA5-4404-9771-E51F1A78CCAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3DCBC87-226F-4D83-ADFE-2178829A4AE4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A8D88B3-F603-4313-AC14-F1B2905698D7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59A15667-1AA5-4404-9771-E51F1A78CCAA}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3DCBC87-226F-4D83-ADFE-2178829A4AE4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="f95d585e-e7a7-414c-955d-38a47c8579bd"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="33ab045e-9213-4eea-a9f2-a5b809105d1e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A8D88B3-F603-4313-AC14-F1B2905698D7}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>